<commit_message>
Update .gitignore, enhance Adidas scraper with additional search URLs, and modify Excel export logic
</commit_message>
<xml_diff>
--- a/port.xlsx
+++ b/port.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="128">
   <si>
     <t>External ID</t>
   </si>
@@ -28,328 +28,376 @@
     <t>Variant Image</t>
   </si>
   <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889652351</t>
-  </si>
-  <si>
-    <t>ID6166</t>
-  </si>
-  <si>
-    <t>size: 5-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889652313</t>
-  </si>
-  <si>
-    <t>size: 4-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889680248</t>
-  </si>
-  <si>
-    <t>size: 6</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889652276</t>
-  </si>
-  <si>
-    <t>size: 7</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889680255</t>
-  </si>
-  <si>
-    <t>size: 4</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889652269</t>
-  </si>
-  <si>
-    <t>size: 5</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889652337</t>
-  </si>
-  <si>
-    <t>size: 6-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6166_nofit_ADULT_FEMALE_4067889652283</t>
-  </si>
-  <si>
-    <t>size: 7-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6528_nofit_ADULT_MEN_4067888588217</t>
-  </si>
-  <si>
-    <t>ID6528</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6528_nofit_ADULT_MEN_4067888588088</t>
-  </si>
-  <si>
-    <t>size: 8</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6528_nofit_ADULT_MEN_4067888588224</t>
-  </si>
-  <si>
-    <t>size: 9</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6528_nofit_ADULT_MEN_4067888588170</t>
-  </si>
-  <si>
-    <t>size: 10</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6528_nofit_ADULT_MEN_4067888588187</t>
-  </si>
-  <si>
-    <t>size: 11</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID6528_nofit_ADULT_MEN_4067888588200</t>
-  </si>
-  <si>
-    <t>size: 12</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832307</t>
-  </si>
-  <si>
-    <t>ID8633</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832369</t>
-  </si>
-  <si>
-    <t>size: 3-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832413</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832475</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832420</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832482</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832468</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8633_nofit_ADULT_FEMALE_4067891832444</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889688077</t>
-  </si>
-  <si>
-    <t>ID8812</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889687988</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889687926</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889688091</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889688015</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889687964</t>
-  </si>
-  <si>
-    <t>size: 8-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID8812_nofit_ADULT_MALE_4067889688060</t>
-  </si>
-  <si>
-    <t>size: 9-</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891549</t>
-  </si>
-  <si>
-    <t>ID9047</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891570</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891600</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891518</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891648</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891563</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891501</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9047_nofit_ADULT_UNISEX_4067892891631</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892910776</t>
-  </si>
-  <si>
-    <t>ID9052</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892910783</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892910882</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892910745</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892910769</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892914491</t>
-  </si>
-  <si>
-    <t>_import_.36826_ID9052_nofit_ADULT_UNISEX_4067892910790</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110820</t>
-  </si>
-  <si>
-    <t>IE0525</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110783</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110769</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110790</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110875</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110776</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE0525_nofit_ADULT_MALE_4067889110868</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410016</t>
-  </si>
-  <si>
-    <t>IE1232</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410054</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410061</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410092</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410078</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892406330</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410085</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE1232_nofit_ADULT_UNISEX_4067892410023</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3675_nofit_JUNIOR_KIDS_4067886691544</t>
-  </si>
-  <si>
-    <t>IE3675</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3675_nofit_JUNIOR_KIDS_4067886691568</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3675_nofit_JUNIOR_KIDS_4067886691551</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3675_nofit_JUNIOR_KIDS_4067886691612</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3675_nofit_JUNIOR_KIDS_4067886691582</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3675_nofit_JUNIOR_KIDS_4067886691605</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3676_nofit_JUNIOR_KIDS_4067886691629</t>
-  </si>
-  <si>
-    <t>IE3676</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3676_nofit_JUNIOR_KIDS_4067886695283</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3676_nofit_JUNIOR_KIDS_4067886691643</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3676_nofit_JUNIOR_KIDS_4067886691650</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3676_nofit_JUNIOR_KIDS_4067886691667</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3676_nofit_JUNIOR_KIDS_4067886695276</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3677_nofit_KIDS_UNISEX_4067886695443</t>
-  </si>
-  <si>
-    <t>IE3677</t>
-  </si>
-  <si>
-    <t>size: 1</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3677_nofit_KIDS_UNISEX_4067886695436</t>
-  </si>
-  <si>
-    <t>size: 2-</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3677_nofit_KIDS_UNISEX_4067886695467</t>
-  </si>
-  <si>
-    <t>size: 12-K</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3677_nofit_KIDS_UNISEX_4067886695474</t>
-  </si>
-  <si>
-    <t>size: 13-K</t>
-  </si>
-  <si>
-    <t>_import_.36826_IE3677_nofit_KIDS_UNISEX_4067886695450</t>
-  </si>
-  <si>
-    <t>size: 10K</t>
+    <t>_import_.36826_IN1500_nofit_ADULT_MALE_4067887941457</t>
+  </si>
+  <si>
+    <t>IN1500</t>
+  </si>
+  <si>
+    <t>size: S</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN1500_nofit_ADULT_MALE_4067887941518</t>
+  </si>
+  <si>
+    <t>size: 2XL</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887956727</t>
+  </si>
+  <si>
+    <t>IN1502</t>
+  </si>
+  <si>
+    <t>size: L</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887956741</t>
+  </si>
+  <si>
+    <t>size: M</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887953085</t>
+  </si>
+  <si>
+    <t>size: XL</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887953016</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891095931</t>
+  </si>
+  <si>
+    <t>IN2462</t>
+  </si>
+  <si>
+    <t>size: XS</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099540</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099588</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099557</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099595</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099571</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN5582_nofit_ADULT_MEN_4067893448308</t>
+  </si>
+  <si>
+    <t>IN5582</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN5582_nofit_ADULT_MEN_4067893451315</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN5582_nofit_ADULT_MEN_4067893451339</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277292</t>
+  </si>
+  <si>
+    <t>IN6163</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277315</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277278</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277308</t>
+  </si>
+  <si>
+    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277285</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562516</t>
+  </si>
+  <si>
+    <t>IP3085</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562530</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562554</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562394</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3996_nofit_JUNIOR_UNISEX_4067889406008</t>
+  </si>
+  <si>
+    <t>IP3996</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3996_nofit_JUNIOR_UNISEX_4067889405995</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP3996_nofit_JUNIOR_UNISEX_4067891850875</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854699</t>
+  </si>
+  <si>
+    <t>IP4000</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854729</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854712</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854705</t>
+  </si>
+  <si>
+    <t>_import_.36826_IP9862_nofit_ADULT_UNISEX_4067886275928</t>
+  </si>
+  <si>
+    <t>IP9862</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304511</t>
+  </si>
+  <si>
+    <t>IQ2655</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304481</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304436</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304504</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758662293</t>
+  </si>
+  <si>
+    <t>IQ2958</t>
+  </si>
+  <si>
+    <t>size: 3634</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758662347</t>
+  </si>
+  <si>
+    <t>size: 3334</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758662408</t>
+  </si>
+  <si>
+    <t>size: 3834</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758666024</t>
+  </si>
+  <si>
+    <t>size: 3534</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758666062</t>
+  </si>
+  <si>
+    <t>size: 3034</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887173117</t>
+  </si>
+  <si>
+    <t>IQ3351</t>
+  </si>
+  <si>
+    <t>size: MCD</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887169301</t>
+  </si>
+  <si>
+    <t>size: SAB</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887169431</t>
+  </si>
+  <si>
+    <t>size: MAB</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887173148</t>
+  </si>
+  <si>
+    <t>size: LCD</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887173155</t>
+  </si>
+  <si>
+    <t>size: XLCD</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887169271</t>
+  </si>
+  <si>
+    <t>size: SCD</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854590</t>
+  </si>
+  <si>
+    <t>IQ4040</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854606</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854576</t>
+  </si>
+  <si>
+    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854583</t>
+  </si>
+  <si>
+    <t>_import_.36826_IR6241_nofit_ADULT_UNISEX_4067887832342</t>
+  </si>
+  <si>
+    <t>IR6241</t>
+  </si>
+  <si>
+    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403279</t>
+  </si>
+  <si>
+    <t>IR9534</t>
+  </si>
+  <si>
+    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403446</t>
+  </si>
+  <si>
+    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403354</t>
+  </si>
+  <si>
+    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403309</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887070898</t>
+  </si>
+  <si>
+    <t>IS0379</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887070911</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887067270</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887070867</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887242097</t>
+  </si>
+  <si>
+    <t>IS3732</t>
+  </si>
+  <si>
+    <t>size: XL5"</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887242868</t>
+  </si>
+  <si>
+    <t>size: S 5"</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887242875</t>
+  </si>
+  <si>
+    <t>size: L 5"</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887243681</t>
+  </si>
+  <si>
+    <t>size: M 5"</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887187992</t>
+  </si>
+  <si>
+    <t>IS3809</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887184373</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887184328</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887188074</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887188043</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270090</t>
+  </si>
+  <si>
+    <t>IS4503</t>
+  </si>
+  <si>
+    <t>size: LAB</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270144</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270175</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270274</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887274623</t>
+  </si>
+  <si>
+    <t>size: XLAB</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893103672</t>
+  </si>
+  <si>
+    <t>IS6708</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893103757</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893103740</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893107403</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893107410</t>
+  </si>
+  <si>
+    <t>_import_.36826_IS7049_nofit_ADULT_UNISEX_4067901111958</t>
+  </si>
+  <si>
+    <t>IS7049</t>
   </si>
 </sst>
 </file>
@@ -693,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="30.7109375" customWidth="1"/>
@@ -742,46 +790,46 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D7" s="2"/>
     </row>
@@ -790,22 +838,22 @@
         <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D9" s="2"/>
     </row>
@@ -814,394 +862,392 @@
         <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="D30" s="2"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D31" s="2"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D32" s="2"/>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C33" s="2"/>
       <c r="D33" s="2"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D39" s="2"/>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="D40" s="2"/>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="D41" s="2"/>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="D42" s="2"/>
     </row>
@@ -1210,420 +1256,464 @@
         <v>67</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="D43" s="2"/>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="C44" s="2" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="D44" s="2"/>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="D45" s="2"/>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="D46" s="2"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="D47" s="2"/>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>26</v>
+        <v>79</v>
       </c>
       <c r="D48" s="2"/>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D49" s="2"/>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D50" s="2"/>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="D51" s="2"/>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="D52" s="2"/>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>10</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="C53" s="2"/>
       <c r="D53" s="2"/>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D54" s="2"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D55" s="2"/>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="D56" s="2"/>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="D57" s="2"/>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D58" s="2"/>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="D59" s="2"/>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D60" s="2"/>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D61" s="2"/>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="D62" s="2"/>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="D63" s="2"/>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>14</v>
+        <v>103</v>
       </c>
       <c r="D64" s="2"/>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>16</v>
+        <v>105</v>
       </c>
       <c r="D65" s="2"/>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D66" s="2"/>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D67" s="2"/>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D68" s="2"/>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D69" s="2"/>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D70" s="2"/>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>16</v>
+        <v>114</v>
       </c>
       <c r="D71" s="2"/>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>95</v>
+        <v>113</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="D72" s="2"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="D73" s="2"/>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="D74" s="2"/>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D75" s="2"/>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="D76" s="2"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>111</v>
+        <v>11</v>
       </c>
       <c r="D77" s="2"/>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D78" s="2"/>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D79" s="2"/>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D80" s="2"/>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add additional search URLs to Adidas scraper and update Excel export
</commit_message>
<xml_diff>
--- a/port.xlsx
+++ b/port.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="120">
   <si>
     <t>External ID</t>
   </si>
@@ -28,376 +28,352 @@
     <t>Variant Image</t>
   </si>
   <si>
-    <t>_import_.36826_IN1500_nofit_ADULT_MALE_4067887941457</t>
-  </si>
-  <si>
-    <t>IN1500</t>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659511</t>
+  </si>
+  <si>
+    <t>IY9800</t>
+  </si>
+  <si>
+    <t>size: 146</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659566</t>
+  </si>
+  <si>
+    <t>size: 134</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659450</t>
+  </si>
+  <si>
+    <t>size: 176</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659559</t>
+  </si>
+  <si>
+    <t>size: 164</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659542</t>
+  </si>
+  <si>
+    <t>size: 140</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659498</t>
+  </si>
+  <si>
+    <t>size: 128</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9800_nofit_JUNIOR_UNISEX_4067895659467</t>
+  </si>
+  <si>
+    <t>size: 152</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672329</t>
+  </si>
+  <si>
+    <t>IY9805</t>
+  </si>
+  <si>
+    <t>size: 170</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672367</t>
+  </si>
+  <si>
+    <t>size: 158</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672343</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672381</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672404</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672282</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672305</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895672398</t>
+  </si>
+  <si>
+    <t>_import_.36826_IY9805_nofit_JUNIOR_UNISEX_4067895674125</t>
+  </si>
+  <si>
+    <t>_import_.36826_IZ1778_nofit_ADULT_UNISEX_4067894070218</t>
+  </si>
+  <si>
+    <t>IZ1778</t>
+  </si>
+  <si>
+    <t>_import_.36826_IZ1907_nofit_ADULT_UNISEX_4067896894188</t>
+  </si>
+  <si>
+    <t>IZ1907</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5230_nofit_ADULT_MEN_4067891699818</t>
+  </si>
+  <si>
+    <t>JC5230</t>
+  </si>
+  <si>
+    <t>size: L</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5230_nofit_ADULT_MEN_4067891699863</t>
   </si>
   <si>
     <t>size: S</t>
   </si>
   <si>
-    <t>_import_.36826_IN1500_nofit_ADULT_MALE_4067887941518</t>
+    <t>_import_.36826_JC5230_nofit_ADULT_MEN_4067891699900</t>
+  </si>
+  <si>
+    <t>size: XL</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5230_nofit_ADULT_MEN_4067891699825</t>
+  </si>
+  <si>
+    <t>size: M</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5338_nofit_ADULT_MALE_4067905751754</t>
+  </si>
+  <si>
+    <t>JC5338</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5338_nofit_ADULT_MALE_4067905751785</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5338_nofit_ADULT_MALE_4067905747887</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5338_nofit_ADULT_MALE_4067905747870</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5338_nofit_ADULT_MALE_4067905751761</t>
   </si>
   <si>
     <t>size: 2XL</t>
   </si>
   <si>
-    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887956727</t>
-  </si>
-  <si>
-    <t>IN1502</t>
-  </si>
-  <si>
-    <t>size: L</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887956741</t>
-  </si>
-  <si>
-    <t>size: M</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887953085</t>
-  </si>
-  <si>
-    <t>size: XL</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN1502_nofit_ADULT_MALE_4067887953016</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891095931</t>
-  </si>
-  <si>
-    <t>IN2462</t>
+    <t>_import_.36826_JC5339_nofit_ADULT_MALE_4067905755547</t>
+  </si>
+  <si>
+    <t>JC5339</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5339_nofit_ADULT_MALE_4067905755691</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5339_nofit_ADULT_MALE_4067905755523</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5339_nofit_ADULT_MALE_4067905759330</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5339_nofit_ADULT_MALE_4067905755615</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5340_nofit_ADULT_MALE_4067905766994</t>
+  </si>
+  <si>
+    <t>JC5340</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5340_nofit_ADULT_MALE_4067905767021</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5340_nofit_ADULT_MALE_4067905763245</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5340_nofit_ADULT_MALE_4067905759507</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5340_nofit_ADULT_MALE_4067905767045</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5454_nofit_ADULT_FEMALE_4067887599337</t>
+  </si>
+  <si>
+    <t>JC5454</t>
+  </si>
+  <si>
+    <t>color: REG</t>
   </si>
   <si>
     <t>size: XS</t>
   </si>
   <si>
-    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099540</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099588</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099557</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099595</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN2462_nofit_ADULT_FEMALE_4067891099571</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN5582_nofit_ADULT_MEN_4067893448308</t>
-  </si>
-  <si>
-    <t>IN5582</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN5582_nofit_ADULT_MEN_4067893451315</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN5582_nofit_ADULT_MEN_4067893451339</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277292</t>
-  </si>
-  <si>
-    <t>IN6163</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277315</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277278</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277308</t>
-  </si>
-  <si>
-    <t>_import_.36826_IN6163_nofit_ADULT_MALE_4067905277285</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562516</t>
-  </si>
-  <si>
-    <t>IP3085</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562530</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562554</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3085_nofit_ADULT_WOMEN_4066759562394</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3996_nofit_JUNIOR_UNISEX_4067889406008</t>
-  </si>
-  <si>
-    <t>IP3996</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3996_nofit_JUNIOR_UNISEX_4067889405995</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP3996_nofit_JUNIOR_UNISEX_4067891850875</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854699</t>
-  </si>
-  <si>
-    <t>IP4000</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854729</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854712</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP4000_nofit_ADULT_UNISEX_4067891854705</t>
-  </si>
-  <si>
-    <t>_import_.36826_IP9862_nofit_ADULT_UNISEX_4067886275928</t>
-  </si>
-  <si>
-    <t>IP9862</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304511</t>
-  </si>
-  <si>
-    <t>IQ2655</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304481</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304436</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2655_nofit_ADULT_WOMEN_4067887304504</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758662293</t>
-  </si>
-  <si>
-    <t>IQ2958</t>
-  </si>
-  <si>
-    <t>size: 3634</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758662347</t>
-  </si>
-  <si>
-    <t>size: 3334</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758662408</t>
-  </si>
-  <si>
-    <t>size: 3834</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758666024</t>
-  </si>
-  <si>
-    <t>size: 3534</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ2958_nofit_ADULT_MEN_4066758666062</t>
-  </si>
-  <si>
-    <t>size: 3034</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887173117</t>
-  </si>
-  <si>
-    <t>IQ3351</t>
-  </si>
-  <si>
-    <t>size: MCD</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887169301</t>
-  </si>
-  <si>
-    <t>size: SAB</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887169431</t>
-  </si>
-  <si>
-    <t>size: MAB</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887173148</t>
-  </si>
-  <si>
-    <t>size: LCD</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887173155</t>
-  </si>
-  <si>
-    <t>size: XLCD</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ3351_nofit_ADULT_WOMEN_4067887169271</t>
-  </si>
-  <si>
-    <t>size: SCD</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854590</t>
-  </si>
-  <si>
-    <t>IQ4040</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854606</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854576</t>
-  </si>
-  <si>
-    <t>_import_.36826_IQ4040_nofit_ADULT_UNISEX_4067891854583</t>
-  </si>
-  <si>
-    <t>_import_.36826_IR6241_nofit_ADULT_UNISEX_4067887832342</t>
-  </si>
-  <si>
-    <t>IR6241</t>
-  </si>
-  <si>
-    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403279</t>
-  </si>
-  <si>
-    <t>IR9534</t>
-  </si>
-  <si>
-    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403446</t>
-  </si>
-  <si>
-    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403354</t>
-  </si>
-  <si>
-    <t>_import_.36826_IR9534_nofit_ADULT_FEMALE_4066757403309</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887070898</t>
-  </si>
-  <si>
-    <t>IS0379</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887070911</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887067270</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS0379_nofit_ADULT_FEMALE_4067887070867</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887242097</t>
-  </si>
-  <si>
-    <t>IS3732</t>
-  </si>
-  <si>
-    <t>size: XL5"</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887242868</t>
-  </si>
-  <si>
-    <t>size: S 5"</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887242875</t>
-  </si>
-  <si>
-    <t>size: L 5"</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3732_nofit_ADULT_MEN_4067887243681</t>
-  </si>
-  <si>
-    <t>size: M 5"</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887187992</t>
-  </si>
-  <si>
-    <t>IS3809</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887184373</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887184328</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887188074</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS3809_nofit_ADULT_MALE_4067887188043</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270090</t>
-  </si>
-  <si>
-    <t>IS4503</t>
-  </si>
-  <si>
-    <t>size: LAB</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270144</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270175</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887270274</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS4503_nofit_ADULT_FEMALE_4067887274623</t>
-  </si>
-  <si>
-    <t>size: XLAB</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893103672</t>
-  </si>
-  <si>
-    <t>IS6708</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893103757</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893103740</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893107403</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS6708_nofit_ADULT_FEMALE_4067893107410</t>
-  </si>
-  <si>
-    <t>_import_.36826_IS7049_nofit_ADULT_UNISEX_4067901111958</t>
-  </si>
-  <si>
-    <t>IS7049</t>
+    <t>_import_.36826_JC5454_nofit_ADULT_FEMALE_4067887544672</t>
+  </si>
+  <si>
+    <t>color: BLACK</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5454_nofit_ADULT_FEMALE_4067887599269</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5454_nofit_ADULT_FEMALE_4067887599184</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5454_nofit_ADULT_FEMALE_4067887544634</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5724_nofit_ADULT_FEMALE_4067891018701</t>
+  </si>
+  <si>
+    <t>JC5724</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5724_nofit_ADULT_FEMALE_4067891018695</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5724_nofit_ADULT_FEMALE_4067891018718</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5724_nofit_ADULT_FEMALE_4067891018657</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5724_nofit_ADULT_FEMALE_4067891018671</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5724_nofit_ADULT_FEMALE_4067891018688</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5728_nofit_ADULT_FEMALE_4067891020957</t>
+  </si>
+  <si>
+    <t>JC5728</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5728_nofit_ADULT_FEMALE_4067891020896</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5728_nofit_ADULT_FEMALE_4067891020926</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5728_nofit_ADULT_FEMALE_4067891020919</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5728_nofit_ADULT_FEMALE_4067891020940</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5728_nofit_ADULT_FEMALE_4067891020933</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5733_nofit_ADULT_FEMALE_4067891022395</t>
+  </si>
+  <si>
+    <t>JC5733</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5733_nofit_ADULT_FEMALE_4067891022388</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5733_nofit_ADULT_FEMALE_4067891022432</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5733_nofit_ADULT_FEMALE_4067891022371</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5733_nofit_ADULT_FEMALE_4067891022418</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5944_nofit_ADULT_FEMALE_4067905791897</t>
+  </si>
+  <si>
+    <t>JC5944</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5944_nofit_ADULT_FEMALE_4067905788071</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5944_nofit_ADULT_FEMALE_4067905791880</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5944_nofit_ADULT_FEMALE_4067905791705</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5944_nofit_ADULT_FEMALE_4067905791729</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5944_nofit_ADULT_FEMALE_4067905791781</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5946_nofit_ADULT_FEMALE_4067902832616</t>
+  </si>
+  <si>
+    <t>JC5946</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5946_nofit_ADULT_FEMALE_4067902832579</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5946_nofit_ADULT_FEMALE_4067902835709</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5946_nofit_ADULT_FEMALE_4067902832555</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5946_nofit_ADULT_FEMALE_4067902835662</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5946_nofit_ADULT_FEMALE_4067902832593</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5960_nofit_ADULT_FEMALE_4067891005893</t>
+  </si>
+  <si>
+    <t>JC5960</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5960_nofit_ADULT_FEMALE_4067891005817</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5960_nofit_ADULT_FEMALE_4067891005855</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5960_nofit_ADULT_FEMALE_4067891009587</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5960_nofit_ADULT_FEMALE_4067891005794</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC5960_nofit_ADULT_FEMALE_4067891005886</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC6025_nofit_ADULT_UNISEX_4067891652707</t>
+  </si>
+  <si>
+    <t>JC6025</t>
+  </si>
+  <si>
+    <t>size: OSFW</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC6025_nofit_ADULT_UNISEX_4067891652714</t>
+  </si>
+  <si>
+    <t>size: OSFM</t>
+  </si>
+  <si>
+    <t>_import_.36826_JC6037_nofit_ADULT_UNISEX_4067891660269</t>
+  </si>
+  <si>
+    <t>JC6037</t>
   </si>
 </sst>
 </file>
@@ -741,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="30.7109375" customWidth="1"/>
@@ -790,46 +766,46 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="D7" s="2"/>
     </row>
@@ -838,118 +814,118 @@
         <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D17" s="2"/>
     </row>
@@ -958,762 +934,804 @@
         <v>31</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C18" s="2"/>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>15</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="C19" s="2"/>
       <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="D30" s="2"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="D31" s="2"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="D32" s="2"/>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C33" s="2"/>
       <c r="D33" s="2"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D39" s="2"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>57</v>
-      </c>
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
       <c r="C40" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D40" s="2"/>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D41" s="2"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>57</v>
-      </c>
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
       <c r="C42" s="2" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="D42" s="2"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="D43" s="2"/>
     </row>
     <row r="44" spans="1:4">
-      <c r="A44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
       <c r="C44" s="2" t="s">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="D44" s="2"/>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="D45" s="2"/>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
       <c r="C46" s="2" t="s">
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="D46" s="2"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="D47" s="2"/>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
       <c r="C48" s="2" t="s">
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="D48" s="2"/>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="D49" s="2"/>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D50" s="2"/>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D51" s="2"/>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="D52" s="2"/>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="2" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C53" s="2"/>
+        <v>73</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="D53" s="2"/>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="2" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="D54" s="2"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>13</v>
+        <v>66</v>
       </c>
       <c r="D55" s="2"/>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="2" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D56" s="2"/>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="2" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D57" s="2"/>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="2" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D58" s="2"/>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="2" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="D59" s="2"/>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="2" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="D60" s="2"/>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="2" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D61" s="2"/>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="2" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>99</v>
+        <v>43</v>
       </c>
       <c r="D62" s="2"/>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="2" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="D63" s="2"/>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="2" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>103</v>
+        <v>39</v>
       </c>
       <c r="D64" s="2"/>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="2" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="D65" s="2"/>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="2" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="D66" s="2"/>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="2" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="D67" s="2"/>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="2" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="D68" s="2"/>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="2" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="D69" s="2"/>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="2" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="D70" s="2"/>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="2" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="D71" s="2"/>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="2" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D72" s="2"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="2" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="D73" s="2"/>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="2" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="D74" s="2"/>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="2" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>119</v>
+        <v>41</v>
       </c>
       <c r="D75" s="2"/>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="2" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D76" s="2"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="2" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="D77" s="2"/>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" s="2" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>13</v>
+        <v>66</v>
       </c>
       <c r="D78" s="2"/>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" s="2" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D79" s="2"/>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="2" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D80" s="2"/>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C81" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="D81" s="2"/>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D82" s="2"/>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D83" s="2"/>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D84" s="2"/>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D85" s="2"/>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D86" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>